<commit_message>
Use supplied official document templates unchanged
</commit_message>
<xml_diff>
--- a/public/templates/HF-yeni.xlsx
+++ b/public/templates/HF-yeni.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
+    <workbookView minimized="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="41">
   <si>
     <t xml:space="preserve">Bakı şəhəri   </t>
   </si>
@@ -113,9 +113,6 @@
     <t>Ümumi dəyəri</t>
   </si>
   <si>
-    <t>kq</t>
-  </si>
-  <si>
     <t>Cəm</t>
   </si>
   <si>
@@ -184,26 +181,32 @@
     </r>
   </si>
   <si>
-    <t>AzRosPromİnvest</t>
-  </si>
-  <si>
-    <t>Şayba M24 (yaylı)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Şayba M24 </t>
-  </si>
-  <si>
-    <t>Bolt M24x100 (qara)</t>
-  </si>
-  <si>
-    <t>Qayka M24</t>
+    <t>BRONZ KEÇİD TESCO</t>
+  </si>
+  <si>
+    <t>ədəd</t>
+  </si>
+  <si>
+    <t>334.08</t>
+  </si>
+  <si>
+    <t>2190.08</t>
+  </si>
+  <si>
+    <t>ACG  BUSİNESS AVİATİON</t>
+  </si>
+  <si>
+    <t>BEYNƏLXALQ AEROPRT</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 04.09.2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -284,6 +287,28 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Droid Sans"/>
     </font>
   </fonts>
   <fills count="2">
@@ -360,20 +385,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -381,45 +397,63 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -867,97 +901,97 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="11"/>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
+      <c r="A1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="11"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="11"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
+      <c r="A5" s="14"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="11"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
+      <c r="A6" s="14"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="11"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
+      <c r="A7" s="14"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
     </row>
     <row r="9" spans="1:7" ht="18.5">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="17"/>
-      <c r="F9" s="21">
-        <v>46250</v>
-      </c>
-      <c r="G9" s="12"/>
+      <c r="B9" s="10"/>
+      <c r="F9" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9" s="16"/>
     </row>
     <row r="12" spans="1:7" ht="14.5" customHeight="1">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
     </row>
     <row r="13" spans="1:7" ht="14.5" customHeight="1">
-      <c r="A13" s="16"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
     </row>
     <row r="14" spans="1:7" ht="14.5" customHeight="1">
       <c r="A14" s="1" t="s">
@@ -967,12 +1001,12 @@
         <v>7</v>
       </c>
       <c r="C14" s="20"/>
-      <c r="D14" s="3"/>
+      <c r="D14" s="21"/>
       <c r="E14" s="2" t="s">
         <v>3</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G14" s="20"/>
     </row>
@@ -984,11 +1018,13 @@
         <v>5</v>
       </c>
       <c r="C15" s="20"/>
-      <c r="D15" s="3"/>
+      <c r="D15" s="21"/>
       <c r="E15" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F15" s="19"/>
+      <c r="F15" s="19" t="s">
+        <v>39</v>
+      </c>
       <c r="G15" s="20"/>
     </row>
     <row r="16" spans="1:7" ht="14.5" customHeight="1">
@@ -999,276 +1035,228 @@
         <v>8</v>
       </c>
       <c r="C16" s="20"/>
-      <c r="D16" s="3"/>
+      <c r="D16" s="21"/>
       <c r="E16" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F16" s="19"/>
       <c r="G16" s="20"/>
     </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="22"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="22"/>
+    </row>
     <row r="18" spans="1:7" ht="29" customHeight="1">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="B18" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="18"/>
-      <c r="D18" s="4" t="s">
+      <c r="C18" s="11"/>
+      <c r="D18" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F18" s="5" t="s">
+      <c r="F18" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="8" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:7">
-      <c r="A19" s="6">
+      <c r="A19" s="7">
         <v>1</v>
       </c>
-      <c r="B19" s="15" t="s">
+      <c r="B19" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19" s="12"/>
+      <c r="D19" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E19" s="6">
+        <v>1</v>
+      </c>
+      <c r="F19" s="6">
+        <v>1856</v>
+      </c>
+      <c r="G19" s="6">
+        <v>1856</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="18"/>
+      <c r="B20" s="18"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G20" s="6">
+        <v>1856</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="18"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G21" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C19" s="15"/>
-      <c r="D19" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E19" s="22">
-        <v>1.3</v>
-      </c>
-      <c r="F19" s="22">
-        <v>5</v>
-      </c>
-      <c r="G19" s="22">
-        <v>6.5</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20" s="6">
-        <v>2</v>
-      </c>
-      <c r="B20" s="15" t="s">
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="18"/>
+      <c r="B22" s="18"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G22" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E20" s="22">
-        <v>1.7</v>
-      </c>
-      <c r="F20" s="22">
-        <v>5</v>
-      </c>
-      <c r="G20" s="22">
-        <v>8.5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" s="6">
-        <v>3</v>
-      </c>
-      <c r="B21" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="C21" s="15"/>
-      <c r="D21" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E21" s="22">
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="E23" s="4"/>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="E24" s="4"/>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="E25" s="4"/>
+    </row>
+    <row r="27" spans="1:7" ht="14" customHeight="1">
+      <c r="A27" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="B27" s="24"/>
+      <c r="C27" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="D27" s="25"/>
+      <c r="E27" s="25"/>
+    </row>
+    <row r="28" spans="1:7" ht="14" customHeight="1">
+      <c r="A28" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="B28" s="24"/>
+      <c r="C28" s="26">
+        <v>1605987621</v>
+      </c>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
+    </row>
+    <row r="29" spans="1:7" ht="14" customHeight="1">
+      <c r="A29" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="F21" s="22">
-        <v>8</v>
-      </c>
-      <c r="G21" s="22">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" s="6">
-        <v>4</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E22" s="22">
-        <v>5</v>
-      </c>
-      <c r="F22" s="22">
-        <v>8</v>
-      </c>
-      <c r="G22" s="22">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="G23" s="22">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
-      <c r="A24" s="7"/>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="G24" s="22">
-        <v>38.700000000000003</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25" s="7"/>
-      <c r="B25" s="7"/>
-      <c r="C25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G25" s="22">
-        <v>253.7</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="14" customHeight="1">
-      <c r="A27" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B27" s="13"/>
-      <c r="C27" s="9" t="s">
+      <c r="B29" s="24"/>
+      <c r="C29" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="D29" s="26"/>
+      <c r="E29" s="26"/>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B30" s="24"/>
+      <c r="C30" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="D30" s="25"/>
+      <c r="E30" s="25"/>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="B31" s="24"/>
+      <c r="C31" s="25">
+        <v>9900003611</v>
+      </c>
+      <c r="D31" s="25"/>
+      <c r="E31" s="25"/>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="B32" s="24"/>
+      <c r="C32" s="26">
+        <v>201229</v>
+      </c>
+      <c r="D32" s="26"/>
+      <c r="E32" s="26"/>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="B33" s="24"/>
+      <c r="C33" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-    </row>
-    <row r="28" spans="1:7" ht="14" customHeight="1">
-      <c r="A28" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="B28" s="13"/>
-      <c r="C28" s="10">
-        <v>1605987621</v>
-      </c>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-    </row>
-    <row r="29" spans="1:7" ht="14" customHeight="1">
-      <c r="A29" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B29" s="13"/>
-      <c r="C29" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-    </row>
-    <row r="30" spans="1:7">
-      <c r="A30" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="B30" s="13"/>
-      <c r="C30" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-    </row>
-    <row r="31" spans="1:7">
-      <c r="A31" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="B31" s="13"/>
-      <c r="C31" s="9">
-        <v>9900003611</v>
-      </c>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-    </row>
-    <row r="32" spans="1:7">
-      <c r="A32" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="B32" s="13"/>
-      <c r="C32" s="10">
-        <v>201229</v>
-      </c>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-    </row>
-    <row r="33" spans="1:5">
-      <c r="A33" s="13" t="s">
+      <c r="D33" s="25"/>
+      <c r="E33" s="25"/>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B33" s="13"/>
-      <c r="C33" s="9" t="s">
+      <c r="B34" s="24"/>
+      <c r="C34" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="D34" s="25"/>
+      <c r="E34" s="25"/>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="B35" s="25"/>
+      <c r="C35" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="D35" s="26"/>
+      <c r="E35" s="26"/>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="D39" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D33" s="9"/>
-      <c r="E33" s="9"/>
-    </row>
-    <row r="34" spans="1:5">
-      <c r="A34" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B34" s="13"/>
-      <c r="C34" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
-    </row>
-    <row r="35" spans="1:5">
-      <c r="A35" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="B35" s="14"/>
-      <c r="C35" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-    </row>
-    <row r="39" spans="1:5">
-      <c r="D39" s="8" t="s">
-        <v>34</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="33">
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="A12:G13"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F15:G15"/>
+  <mergeCells count="30">
+    <mergeCell ref="A35:B35"/>
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="C33:E33"/>
     <mergeCell ref="C34:E34"/>
@@ -1285,7 +1273,19 @@
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="A12:G13"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F15:G15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>